<commit_message>
avance de la pagina
</commit_message>
<xml_diff>
--- a/docs/DSY1104 - Forma C - Catalogo Distribuidora Gas El Volcan.xlsx
+++ b/docs/DSY1104 - Forma C - Catalogo Distribuidora Gas El Volcan.xlsx
@@ -347,27 +347,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -397,19 +383,19 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" quotePrefix="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" quotePrefix="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" quotePrefix="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" quotePrefix="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" quotePrefix="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" quotePrefix="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" quotePrefix="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" quotePrefix="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" quotePrefix="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" quotePrefix="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" quotePrefix="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -489,10 +475,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;#xFF2D;&amp;#xFF33; &amp;#xFF30;&amp;#x30B4;&amp;#x30B7;&amp;#x30C3;&amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;#xB9D1;&amp;#xC740; &amp;#xACE0;&amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;#x5B8B;&amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;#x65B0;&amp;#x7D30;&amp;#x660E;&amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;#xFF2D;&amp;amp;#xFF33; &amp;amp;#xFF30;&amp;amp;#x30B4;&amp;amp;#x30B7;&amp;amp;#x30C3;&amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;#xB9D1;&amp;amp;#xC740; &amp;amp;#xACE0;&amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;#x5B8B;&amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;#x65B0;&amp;amp;#x7D30;&amp;amp;#x660E;&amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -523,10 +509,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;#xFF2D;&amp;#xFF33; &amp;#xFF30;&amp;#x30B4;&amp;#x30B7;&amp;#x30C3;&amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;#xB9D1;&amp;#xC740; &amp;#xACE0;&amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;#x5B8B;&amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;#x65B0;&amp;#x7D30;&amp;#x660E;&amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;#xFF2D;&amp;amp;#xFF33; &amp;amp;#xFF30;&amp;amp;#x30B4;&amp;amp;#x30B7;&amp;amp;#x30C3;&amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;#xB9D1;&amp;amp;#xC740; &amp;amp;#xACE0;&amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;#x5B8B;&amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;#x65B0;&amp;amp;#x7D30;&amp;amp;#x660E;&amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -727,7 +713,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{73964287-FD7F-41FB-8B6B-834B5C646E7C}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{340E3C41-8985-48C1-8BE0-93C7D2CF30D8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -1148,7 +1134,7 @@
   </mergeCells>
   <printOptions/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
@@ -1158,7 +1144,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{CAD9F565-A496-46B9-99DC-11FFE17C09A1}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D88CB62D-F477-4D79-B656-7B82A29323E3}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -1287,7 +1273,7 @@
   </mergeCells>
   <printOptions/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>

</xml_diff>

<commit_message>
catalogo de el volcan
</commit_message>
<xml_diff>
--- a/docs/DSY1104 - Forma C - Catalogo Distribuidora Gas El Volcan.xlsx
+++ b/docs/DSY1104 - Forma C - Catalogo Distribuidora Gas El Volcan.xlsx
@@ -475,10 +475,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;amp;amp;amp;#xFF2D;&amp;amp;amp;amp;#xFF33; &amp;amp;amp;amp;#xFF30;&amp;amp;amp;amp;#x30B4;&amp;amp;amp;amp;#x30B7;&amp;amp;amp;amp;#x30C3;&amp;amp;amp;amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;amp;amp;amp;#xB9D1;&amp;amp;amp;amp;#xC740; &amp;amp;amp;amp;#xACE0;&amp;amp;amp;amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;amp;amp;amp;#x5B8B;&amp;amp;amp;amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;amp;amp;amp;#x65B0;&amp;amp;amp;amp;#x7D30;&amp;amp;amp;amp;#x660E;&amp;amp;amp;amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;amp;amp;amp;#xFF2D;&amp;amp;amp;amp;amp;#xFF33; &amp;amp;amp;amp;amp;#xFF30;&amp;amp;amp;amp;amp;#x30B4;&amp;amp;amp;amp;amp;#x30B7;&amp;amp;amp;amp;amp;#x30C3;&amp;amp;amp;amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;amp;amp;amp;#xB9D1;&amp;amp;amp;amp;amp;#xC740; &amp;amp;amp;amp;amp;#xACE0;&amp;amp;amp;amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;amp;amp;amp;#x5B8B;&amp;amp;amp;amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;amp;amp;amp;#x65B0;&amp;amp;amp;amp;amp;#x7D30;&amp;amp;amp;amp;amp;#x660E;&amp;amp;amp;amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -509,10 +509,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="&amp;amp;amp;amp;#xFF2D;&amp;amp;amp;amp;#xFF33; &amp;amp;amp;amp;#xFF30;&amp;amp;amp;amp;#x30B4;&amp;amp;amp;amp;#x30B7;&amp;amp;amp;amp;#x30C3;&amp;amp;amp;amp;#x30AF;"/>
-        <a:font script="Hang" typeface="&amp;amp;amp;amp;#xB9D1;&amp;amp;amp;amp;#xC740; &amp;amp;amp;amp;#xACE0;&amp;amp;amp;amp;#xB515;"/>
-        <a:font script="Hans" typeface="&amp;amp;amp;amp;#x5B8B;&amp;amp;amp;amp;#x4F53;"/>
-        <a:font script="Hant" typeface="&amp;amp;amp;amp;#x65B0;&amp;amp;amp;amp;#x7D30;&amp;amp;amp;amp;#x660E;&amp;amp;amp;amp;#x9AD4;"/>
+        <a:font script="Jpan" typeface="&amp;amp;amp;amp;amp;#xFF2D;&amp;amp;amp;amp;amp;#xFF33; &amp;amp;amp;amp;amp;#xFF30;&amp;amp;amp;amp;amp;#x30B4;&amp;amp;amp;amp;amp;#x30B7;&amp;amp;amp;amp;amp;#x30C3;&amp;amp;amp;amp;amp;#x30AF;"/>
+        <a:font script="Hang" typeface="&amp;amp;amp;amp;amp;#xB9D1;&amp;amp;amp;amp;amp;#xC740; &amp;amp;amp;amp;amp;#xACE0;&amp;amp;amp;amp;amp;#xB515;"/>
+        <a:font script="Hans" typeface="&amp;amp;amp;amp;amp;#x5B8B;&amp;amp;amp;amp;amp;#x4F53;"/>
+        <a:font script="Hant" typeface="&amp;amp;amp;amp;amp;#x65B0;&amp;amp;amp;amp;amp;#x7D30;&amp;amp;amp;amp;amp;#x660E;&amp;amp;amp;amp;amp;#x9AD4;"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -713,7 +713,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{A1C67A04-CE6E-45C6-8185-DE35FFD9879B}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{86AAE489-9E83-430F-8431-F8DD5924FDFA}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -1144,7 +1144,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{9F14E80B-6AB0-4895-8A98-3E8A8362EE0B}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D5079DBF-A066-4C86-BC85-C4199C2D5667}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>

</xml_diff>